<commit_message>
add amistoso vs Nazca individual 37min
</commit_message>
<xml_diff>
--- a/Matches.xlsx
+++ b/Matches.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="PfSSf3eX/0LJpb4lXO3mWilv2huS1nI0WF8HSSC52kI="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="9aXg8AtziO2Ca8XrTZ1EuBgYu218exaxgW879T92pY0="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>fecha</t>
   </si>
@@ -63,31 +63,16 @@
     <t>Propio</t>
   </si>
   <si>
-    <t>https://youtu.be/ivunOFSM1ME</t>
+    <t>https://youtu.be/Xk6znucIHM8</t>
   </si>
   <si>
     <t>Entrenamiento</t>
   </si>
   <si>
-    <t>SV Max Uhle</t>
-  </si>
-  <si>
-    <t>AD Strangers</t>
-  </si>
-  <si>
-    <t>Trabajo principal</t>
-  </si>
-  <si>
-    <t>https://youtu.be/n5sBx_cosTY</t>
-  </si>
-  <si>
-    <t>Parte 1 Trabajo previo</t>
-  </si>
-  <si>
-    <t>https://youtu.be/X55mwKhQgTI</t>
-  </si>
-  <si>
-    <t>Parte 2 Trabajo previo</t>
+    <t>Sporting Company</t>
+  </si>
+  <si>
+    <t>Santos FC</t>
   </si>
 </sst>
 </file>
@@ -117,19 +102,16 @@
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
-      <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <u/>
-      <sz val="11.0"/>
-      <color rgb="FF0563C1"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -159,20 +141,17 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -395,7 +374,7 @@
     <col customWidth="1" min="8" max="8" width="17.57"/>
     <col customWidth="1" min="9" max="9" width="14.71"/>
     <col customWidth="1" min="10" max="10" width="9.14"/>
-    <col customWidth="1" min="11" max="11" width="19.0"/>
+    <col customWidth="1" min="11" max="11" width="27.57"/>
     <col customWidth="1" min="12" max="12" width="17.14"/>
     <col customWidth="1" min="13" max="13" width="7.43"/>
     <col customWidth="1" min="14" max="26" width="9.14"/>
@@ -450,81 +429,39 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46087.0</v>
+        <v>46102.0</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="4" t="str">
-        <f t="shared" ref="C2:C4" si="1">CONCATENATE(F2,A2)</f>
-        <v>46087</v>
-      </c>
+      <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="L2" s="7" t="str">
-        <f>CONCATENATE( "vs ",I2)</f>
-        <v>vs AD Strangers</v>
-      </c>
-      <c r="O2" s="7" t="b">
+      <c r="K2" s="7"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="9">
+        <v>0.0</v>
+      </c>
+      <c r="N2" s="9">
+        <v>3.0</v>
+      </c>
+      <c r="O2" s="8" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>46087.0</v>
-      </c>
-      <c r="C3" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>46087</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="O3" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>46087.0</v>
-      </c>
-      <c r="C4" s="4" t="str">
-        <f t="shared" si="1"/>
-        <v>46087</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="O4" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="D5" s="10"/>
-    </row>
+    <row r="12" ht="15.75" customHeight="1"/>
+    <row r="13" ht="15.75" customHeight="1"/>
+    <row r="14" ht="15.75" customHeight="1"/>
+    <row r="15" ht="15.75" customHeight="1"/>
+    <row r="16" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -1500,20 +1437,13 @@
     <row r="989" ht="15.75" customHeight="1"/>
     <row r="990" ht="15.75" customHeight="1"/>
     <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
-    <hyperlink r:id="rId2" ref="D3"/>
-    <hyperlink r:id="rId3" ref="D4"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add entrenamientos y match hasta 27-03
</commit_message>
<xml_diff>
--- a/Matches.xlsx
+++ b/Matches.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>fecha</t>
   </si>
@@ -66,23 +66,30 @@
     <t>https://youtu.be/Xk6znucIHM8</t>
   </si>
   <si>
-    <t>Entrenamiento</t>
+    <t>amistoso</t>
   </si>
   <si>
     <t>Sporting Company</t>
   </si>
   <si>
     <t>Santos FC</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IetP2iEXvv4</t>
+  </si>
+  <si>
+    <t>Nacional de Tinguiña</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -107,11 +114,15 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="2">
@@ -128,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -149,7 +160,13 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -436,26 +453,58 @@
       <c r="E2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="7">
+      <c r="J2" s="6">
         <v>1.0</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="7" t="s">
         <v>18</v>
       </c>
       <c r="L2" s="8"/>
-      <c r="M2" s="7">
+      <c r="M2" s="6">
         <v>0.0</v>
       </c>
-      <c r="N2" s="7">
+      <c r="N2" s="6">
         <v>3.0</v>
       </c>
       <c r="O2" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9">
+        <v>46106.0</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="N3" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="O3" s="8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1442,10 +1491,11 @@
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
+    <hyperlink r:id="rId2" ref="D3"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add data 2T colectivo vs CRISTAL 0204
</commit_message>
<xml_diff>
--- a/Matches.xlsx
+++ b/Matches.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>fecha</t>
   </si>
@@ -79,15 +79,31 @@
   </si>
   <si>
     <t>Nacional de Tinguiña</t>
+  </si>
+  <si>
+    <t>https://youtu.be/0_4O_T7QRPg</t>
+  </si>
+  <si>
+    <t>Universitario</t>
+  </si>
+  <si>
+    <t>Municipal</t>
+  </si>
+  <si>
+    <t>https://youtu.be/8Xf9SK91JKc</t>
+  </si>
+  <si>
+    <t>Sporting Cristal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -139,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -165,6 +181,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -505,6 +524,99 @@
         <v>1.0</v>
       </c>
       <c r="O3" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11">
+        <v>46109.0</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="N4" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="O4" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11">
+        <v>46082.0</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="N5" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="O5" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11">
+        <v>46083.0</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="M6" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="N6" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="O6" s="8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1492,10 +1604,12 @@
   <hyperlinks>
     <hyperlink r:id="rId1" ref="D2"/>
     <hyperlink r:id="rId2" ref="D3"/>
+    <hyperlink r:id="rId3" ref="D4"/>
+    <hyperlink r:id="rId4" ref="D6"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>